<commit_message>
Cosmetic improvement of StreamLit app
Improve bus and signals explorer
</commit_message>
<xml_diff>
--- a/ICD_Database.xlsx
+++ b/ICD_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\SignalCraft\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA955B0-0B0E-4017-923C-A35EAF2B442B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AEBA3A0-56B7-4314-9C5F-DBA7C2C6E816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8588" uniqueCount="2194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8588" uniqueCount="2196">
   <si>
     <t>ICD — Signal database</t>
   </si>
@@ -6648,6 +6648,12 @@
   </si>
   <si>
     <t>1_Signals holds the functional range of a quantity: unit, functional minimum and functional maximum as the interface is expected to behave in service. Bus-definition tabs hold the encoded range, which is usually wider and may use a scaled unit. A pitch limited to 45 deg in service can ride in a field that encodes 90 deg.</t>
+  </si>
+  <si>
+    <t>Power Lever Idle position</t>
+  </si>
+  <si>
+    <t>Power Lever Position backup</t>
   </si>
 </sst>
 </file>
@@ -14267,7 +14273,7 @@
         <v>354</v>
       </c>
       <c r="C9" t="s">
-        <v>355</v>
+        <v>2195</v>
       </c>
       <c r="D9" t="s">
         <v>321</v>
@@ -14314,7 +14320,7 @@
         <v>354</v>
       </c>
       <c r="C10" t="s">
-        <v>355</v>
+        <v>2194</v>
       </c>
       <c r="D10" t="s">
         <v>321</v>

</xml_diff>